<commit_message>
Add floor deck under laminate and drop kitchen from estimate
Laminate sits on 12 mm plywood over UFH plates, not on the plates.
Optional 18 mm OSB if joists are still open under the film.
Kitchen fixtures and GVL on living partitions are out.

Co-authored-by: PavelP78 <PavelP78@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/barnhouse/smeta_barnhouse_mdf.xlsx
+++ b/barnhouse/smeta_barnhouse_mdf.xlsx
@@ -22,7 +22,7 @@
     <sheet name="Прочее" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Смета'!$A$4:$I$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Смета'!$A$4:$I$106</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Смета'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Сводка'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Исходные'!$A$4:$D$19</definedName>
@@ -413,12 +413,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Сводка'!$B$5:$B$15</f>
+              <f>'Сводка'!$B$5:$B$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Сводка'!$C$5:$C$15</f>
+              <f>'Сводка'!$C$5:$C$14</f>
             </numRef>
           </val>
         </ser>
@@ -755,7 +755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -833,7 +833,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1.  Перегородки — заполнение и обшивка каркаса (каркас уже стоит)</t>
+          <t>1.  Перегородки — вата в каркас; лист только в с/у (каркас уже стоит)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -883,7 +883,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>между отапливаемыми комнатами, звукоизоляция</t>
+          <t>звук между комнатами; лист с жилой стороны не кладём</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>ГВЛ / ГСП 12.5 мм на перегородки, 2 стороны</t>
+          <t>ГВЛВ 12.5 мм в с/у (стены + потолок)</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -904,10 +904,10 @@
         </is>
       </c>
       <c r="D7" s="13" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>720</v>
+        <v>890</v>
       </c>
       <c r="F7" s="15">
         <f>IF(D7="","",D7*E7)</f>
@@ -915,17 +915,17 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>S обшивки ≈ 88 м² / 3.0 м² + запас</t>
+          <t>вкладка С_у</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>1200×2500</t>
+          <t>1200×2500 влагостойкий</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>жилые стороны под МДФ, с/у — влагостойкий</t>
+          <t>под плитку и краску потолка; жилые перегородки без ГВЛ</t>
         </is>
       </c>
     </row>
@@ -937,19 +937,19 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>ГВЛВ 10–12 мм дополнительно в с/у</t>
+          <t>Саморезы, лента, шпаклёвка швов — только с/у</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>лист</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>890</v>
+        <v>2200</v>
       </c>
       <c r="F8" s="10">
         <f>IF(D8="","",D8*E8)</f>
@@ -957,17 +957,17 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>стены+потолок с/у</t>
+          <t>норма на мокрую зону</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>1200×2500 влагостойкий</t>
+          <t>Кнауф / аналог</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>под плитку и покраску потолка</t>
+          <t>не на весь дом: МДФ идёт по обрешётке на стойки</t>
         </is>
       </c>
     </row>
@@ -979,19 +979,19 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Профиль / саморезы / лента / шпаклёвка швов</t>
+          <t>Лента уплотнительная и демпфер к перегородкам</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>м.п.</t>
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>6500</v>
+        <v>45</v>
       </c>
       <c r="F9" s="15">
         <f>IF(D9="","",D9*E9)</f>
@@ -999,100 +999,101 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>норма на 90 м² обшивки</t>
+          <t>периметр примыканий</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Кнауф / аналог</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>каркас перегородок уже есть — только крепёж листа</t>
-        </is>
-      </c>
+          <t>поролон / Дихтунгсбанд</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Лента уплотнительная и демпфер к перегородкам</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>м.п.</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="E10" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="F10" s="10">
-        <f>IF(D10="","",D10*E10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>периметр примыканий</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>поролон / Дихтунгсбанд</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="16" t="n"/>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="A10" s="16" t="n"/>
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="17">
-        <f>SUM(F6:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="16" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="17">
+        <f>SUM(F6:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="16" t="n"/>
+      <c r="H10" s="16" t="n"/>
+      <c r="I10" s="16" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2.  Обрешётка и МДФ-панели жилых стен и скатных потолков (с/у и терраса нет)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>2.  Обрешётка и МДФ-панели жилых стен и скатных потолков (с/у и терраса нет)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Панель МДФ Союз Классик дуб альпийский 2600×238×6</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D13" s="13">
+        <f>Обшивка!B9</f>
+        <v/>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>260</v>
+      </c>
+      <c r="F13" s="15">
+        <f>IF(D13="","",D13*E13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>вкладка Обшивка</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>раб. 0,572 м², уп. 8 шт</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>ориентир 260 ₽/шт; Петрович продаёт поштучно, кратно 8</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Панель МДФ Союз Классик дуб альпийский 2600×238×6</t>
+          <t>Брусок 20×40×3000 сухой (обрешётка)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1101,11 +1102,11 @@
         </is>
       </c>
       <c r="D14" s="8">
-        <f>Обшивка!B9</f>
+        <f>Обшивка!B12</f>
         <v/>
       </c>
       <c r="E14" s="9" t="n">
-        <v>260</v>
+        <v>95</v>
       </c>
       <c r="F14" s="10">
         <f>IF(D14="","",D14*E14)</f>
@@ -1118,37 +1119,37 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>раб. 0,572 м², уп. 8 шт</t>
+          <t>шаг 400 мм</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>ориентир 260 ₽/шт; Петрович продаёт поштучно, кратно 8</t>
+          <t>по плёнке нар. стен и по листам перегородок</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Брусок 20×40×3000 сухой (обрешётка)</t>
+          <t>Кляймер №3 с гвоздями (под 6 мм)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>упак 100 шт</t>
         </is>
       </c>
       <c r="D15" s="13">
-        <f>Обшивка!B12</f>
+        <f>CEILING(Обшивка!B13/100,1)</f>
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="F15" s="15">
         <f>IF(D15="","",D15*E15)</f>
@@ -1156,42 +1157,37 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>вкладка Обшивка</t>
+          <t>≈8 шт на панель</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>шаг 400 мм</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>по плёнке нар. стен и по листам перегородок</t>
-        </is>
-      </c>
+          <t>кляймер под 6 мм</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Кляймер №3 с гвоздями (под 6 мм)</t>
+          <t>Саморезы 3.5×35 / скобы степлера 6–8 мм</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>упак 100 шт</t>
-        </is>
-      </c>
-      <c r="D16" s="8">
-        <f>CEILING(Обшивка!B13/100,1)</f>
-        <v/>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>1</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>71</v>
+        <v>2200</v>
       </c>
       <c r="F16" s="10">
         <f>IF(D16="","",D16*E16)</f>
@@ -1199,37 +1195,37 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>≈8 шт на панель</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>кляймер под 6 мм</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="inlineStr"/>
+          <t>обрешётка + панели</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>производитель запрещает жидкие гвозди</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Саморезы 3.5×35 / скобы степлера 6–8 мм</t>
+          <t>Угол МДФ универсальный 2600, дуб альпийский</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D17" s="13" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>2200</v>
+        <v>190</v>
       </c>
       <c r="F17" s="15">
         <f>IF(D17="","",D17*E17)</f>
@@ -1237,25 +1233,25 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>обрешётка + панели</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="inlineStr"/>
-      <c r="I17" s="12" t="inlineStr">
-        <is>
-          <t>производитель запрещает жидкие гвозди</t>
-        </is>
-      </c>
+          <t>внутренние/наружные углы</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Союз в цвет панелей</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.6</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Угол МДФ универсальный 2600, дуб альпийский</t>
+          <t>Галтель / потолочный плинтус МДФ 2600 в цвет</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1264,10 +1260,10 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="F18" s="10">
         <f>IF(D18="","",D18*E18)</f>
@@ -1275,12 +1271,12 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>внутренние/наружные углы</t>
+          <t>периметр жилых + конёк</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Союз в цвет панелей</t>
+          <t>закрывает стык панели 2,60 и стену 2,615</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr"/>
@@ -1288,24 +1284,25 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Галтель / потолочный плинтус МДФ 2600 в цвет</t>
+          <t>Плинтус напольный МДФ 60–80 мм + уголки, в цвет</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="n">
-        <v>22</v>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="D19" s="13">
+        <f>Обшивка!B14</f>
+        <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>170</v>
+        <v>290</v>
       </c>
       <c r="F19" s="15">
         <f>IF(D19="","",D19*E19)</f>
@@ -1313,144 +1310,148 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>периметр жилых + конёк</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>закрывает стык панели 2,60 и стену 2,615</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr"/>
+          <t>периметр жилых − двери</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr"/>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>с/у — плинтус керамический в плитке</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Плинтус напольный МДФ 60–80 мм + уголки, в цвет</t>
+          <t>Нащельник у окон/дверей, расходники</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>м.п.</t>
-        </is>
-      </c>
-      <c r="D20" s="8">
-        <f>Обшивка!B14</f>
-        <v/>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>1</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>290</v>
+        <v>3500</v>
       </c>
       <c r="F20" s="10">
         <f>IF(D20="","",D20*E20)</f>
         <v/>
       </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>периметр жилых − двери</t>
-        </is>
-      </c>
+      <c r="G20" s="7" t="inlineStr"/>
       <c r="H20" s="7" t="inlineStr"/>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>с/у — плинтус керамический в плитке</t>
+          <t>изделия окон и дверей свои, только примыкание</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Нащельник у окон/дверей, расходники</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>3500</v>
-      </c>
-      <c r="F21" s="15">
-        <f>IF(D21="","",D21*E21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="12" t="inlineStr"/>
-      <c r="H21" s="12" t="inlineStr"/>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>изделия окон и дверей свои, только примыкание</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="n"/>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="A21" s="16" t="n"/>
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="17">
-        <f>SUM(F14:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="16" t="n"/>
-      <c r="H22" s="16" t="n"/>
-      <c r="I22" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="17">
+        <f>SUM(F13:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="16" t="n"/>
+      <c r="I21" s="16" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>3.  Тёплый пол сухой по всему дому (пол уже утеплён и под плёнкой)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>3.  Тёплый пол сухой по всему дому (пол уже утеплён и под плёнкой)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Теплораспределительная пластина VALTEC VT.FP.SZ</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D24" s="8">
+        <f>Теплый_пол!B12</f>
+        <v/>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>339</v>
+      </c>
+      <c r="F24" s="10">
+        <f>IF(D24="","",D24*E24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>вкладка Теплый_пол</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>VT.FP.SZ.0125 1000×125</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>кратно 40 шт, шаг 125 мм</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Теплораспределительная пластина VALTEC VT.FP.SZ</t>
+          <t>Труба PEX-a / PERT 16×2 для ТП</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>м</t>
         </is>
       </c>
       <c r="D25" s="13">
-        <f>Теплый_пол!B12</f>
+        <f>Теплый_пол!B14</f>
         <v/>
       </c>
       <c r="E25" s="14" t="n">
-        <v>339</v>
+        <v>82</v>
       </c>
       <c r="F25" s="15">
         <f>IF(D25="","",D25*E25)</f>
@@ -1458,42 +1459,41 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>вкладка Теплый_пол</t>
+          <t>≈8 м/м² + 10%</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>VT.FP.SZ.0125 1000×125</t>
+          <t>бухта 200 м ×2</t>
         </is>
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>кратно 40 шт, шаг 125 мм</t>
+          <t>5–6 контуров до 80 м</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Труба PEX-a / PERT 16×2 для ТП</t>
+          <t>Коллектор в сборе с расходомерами, 7 выходов</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="D26" s="8">
-        <f>Теплый_пол!B14</f>
-        <v/>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>1</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>82</v>
+        <v>18900</v>
       </c>
       <c r="F26" s="10">
         <f>IF(D26="","",D26*E26)</f>
@@ -1501,29 +1501,29 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>≈8 м/м² + 10%</t>
+          <t>Теплый_пол!B15</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>бухта 200 м ×2</t>
+          <t>Valtec / Uponor аналог</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>5–6 контуров до 80 м</t>
+          <t>по числу контуров</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Коллектор в сборе с расходомерами, 7 выходов</t>
+          <t>Шкаф коллекторный встраиваемый</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
@@ -1535,37 +1535,33 @@
         <v>1</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>18900</v>
+        <v>4200</v>
       </c>
       <c r="F27" s="15">
         <f>IF(D27="","",D27*E27)</f>
         <v/>
       </c>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>Теплый_пол!B15</t>
-        </is>
-      </c>
+      <c r="G27" s="12" t="inlineStr"/>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>Valtec / Uponor аналог</t>
+          <t>600–800 мм</t>
         </is>
       </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>по числу контуров</t>
+          <t>в холле / кухне</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Шкаф коллекторный встраиваемый</t>
+          <t>Насосно-смесительный узел для ТП</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1577,7 +1573,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>4200</v>
+        <v>18900</v>
       </c>
       <c r="F28" s="10">
         <f>IF(D28="","",D28*E28)</f>
@@ -1586,74 +1582,70 @@
       <c r="G28" s="7" t="inlineStr"/>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>600–800 мм</t>
+          <t>Valtec Combi / аналог</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>в холле / кухне</t>
+          <t>если котёл без своей погоды</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Насосно-смесительный узел для ТП</t>
+          <t>Евроконус 16×3/4, соединители, отводы</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D29" s="13" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>18900</v>
+        <v>5200</v>
       </c>
       <c r="F29" s="15">
         <f>IF(D29="","",D29*E29)</f>
         <v/>
       </c>
-      <c r="G29" s="12" t="inlineStr"/>
-      <c r="H29" s="12" t="inlineStr">
-        <is>
-          <t>Valtec Combi / аналог</t>
-        </is>
-      </c>
-      <c r="I29" s="12" t="inlineStr">
-        <is>
-          <t>если котёл без своей погоды</t>
-        </is>
-      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>на 7 петель</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr"/>
+      <c r="I29" s="12" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Евроконус 16×3/4, соединители, отводы</t>
+          <t>Демпферная лента 8–10 мм</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>м.п.</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>5200</v>
+        <v>35</v>
       </c>
       <c r="F30" s="10">
         <f>IF(D30="","",D30*E30)</f>
@@ -1661,143 +1653,151 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>на 7 петель</t>
+          <t>периметр комнат</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
-      <c r="I30" s="7" t="inlineStr"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>уже есть плёнка пола — лента к стенам</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Демпферная лента 8–10 мм</t>
+          <t>Скотч алюминиевый / фольгированный</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>м.п.</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D31" s="13" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>35</v>
+        <v>320</v>
       </c>
       <c r="F31" s="15">
         <f>IF(D31="","",D31*E31)</f>
         <v/>
       </c>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>периметр комнат</t>
-        </is>
-      </c>
-      <c r="H31" s="12" t="inlineStr"/>
+      <c r="G31" s="12" t="inlineStr"/>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>50 м</t>
+        </is>
+      </c>
       <c r="I31" s="12" t="inlineStr">
         <is>
-          <t>уже есть плёнка пола — лента к стенам</t>
+          <t>стыки плёнки при монтаже пластин</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>3.8</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Скотч алюминиевый / фольгированный</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>320</v>
-      </c>
-      <c r="F32" s="10">
-        <f>IF(D32="","",D32*E32)</f>
-        <v/>
-      </c>
-      <c r="G32" s="7" t="inlineStr"/>
-      <c r="H32" s="7" t="inlineStr">
-        <is>
-          <t>50 м</t>
-        </is>
-      </c>
-      <c r="I32" s="7" t="inlineStr">
-        <is>
-          <t>стыки плёнки при монтаже пластин</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="16" t="n"/>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="A32" s="16" t="n"/>
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C33" s="16" t="n"/>
-      <c r="D33" s="16" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="17">
-        <f>SUM(F25:F32)</f>
-        <v/>
-      </c>
-      <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
-      <c r="I33" s="16" t="n"/>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="17">
+        <f>SUM(F24:F31)</f>
+        <v/>
+      </c>
+      <c r="G32" s="16" t="n"/>
+      <c r="H32" s="16" t="n"/>
+      <c r="I32" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>4.  Основание пола и финиш (ламинат не на пластины ТП)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="5" t="n"/>
+      <c r="I34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>4.  Финиш пола</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n"/>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>OSB-3 18 мм / фанера ФСФ 18 мм — черновой настил по лагам</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>лист 2500×1250</t>
+        </is>
+      </c>
+      <c r="D35" s="13">
+        <f>CEILING(Полы!B10*1.08/3.125,1)</f>
+        <v/>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F35" s="15">
+        <f>IF(D35="","",D35*E35)</f>
+        <v/>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>весь отапливаемый пол +8%</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>3.125 м²/лист</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>обнулить, если черновой пол уже есть; плёнка сама по себе не основание</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Ламинат 33 кл. / SPC для тёплого пола</t>
+          <t>Саморезы 4.2×55 к лагам</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>м²</t>
-        </is>
-      </c>
-      <c r="D36" s="8">
-        <f>Полы!G5+Полы!G6+Полы!G7+Полы!G8</f>
-        <v/>
+          <t>упак 200 шт</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>4</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>1290</v>
+        <v>420</v>
       </c>
       <c r="F36" s="10">
         <f>IF(D36="","",D36*E36)</f>
@@ -1805,42 +1805,34 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>вкладка Полы, с запасом</t>
-        </is>
-      </c>
-      <c r="H36" s="7" t="inlineStr">
-        <is>
-          <t>толщина 8–10 мм, допуск на ТП</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>жилые + холл</t>
-        </is>
-      </c>
+          <t>черновой настил</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr"/>
+      <c r="I36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Подложка под ламинат для ТП (тонкая)</t>
+          <t>Фанера ФСФ 12 мм поверх пластин ТП — под ламинат</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>м²</t>
+          <t>лист 2500×1250</t>
         </is>
       </c>
       <c r="D37" s="13">
-        <f>Полы!G5+Полы!G6+Полы!G7+Полы!G8</f>
+        <f>CEILING((Полы!G5+Полы!G6+Полы!G7+Полы!G8)/3.125,1)</f>
         <v/>
       </c>
       <c r="E37" s="14" t="n">
-        <v>180</v>
+        <v>2190</v>
       </c>
       <c r="F37" s="15">
         <f>IF(D37="","",D37*E37)</f>
@@ -1848,71 +1840,83 @@
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>вкладка Полы</t>
+          <t>жилые с запасом</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>1–2 мм, не фольгированная толстая</t>
+          <t>3.125 м²/лист</t>
         </is>
       </c>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>не режет тепло</t>
+          <t>на этот слой: подложка 1–2 мм и ламинат</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Подложка-гармошка / плёнка подложка</t>
+          <t>ГВЛВ 10 мм, 2 слоя — пол с/у поверх ТП</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>рул</t>
+          <t>лист 1200×2500</t>
         </is>
       </c>
       <c r="D38" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E38" s="9" t="n">
-        <v>900</v>
+        <v>890</v>
       </c>
       <c r="F38" s="10">
         <f>IF(D38="","",D38*E38)</f>
         <v/>
       </c>
-      <c r="G38" s="7" t="inlineStr"/>
-      <c r="H38" s="7" t="inlineStr"/>
-      <c r="I38" s="7" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>3.59 м² ×2 слоя + запас</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>3.0 м²/лист</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>под гидроизоляцию и плитку</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Пороги / стык ламинат–плитка</t>
+          <t>Саморезы 3.5×41 + клей по дереву на настил 12 мм</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D39" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" s="14" t="n">
-        <v>650</v>
+        <v>2800</v>
       </c>
       <c r="F39" s="15">
         <f>IF(D39="","",D39*E39)</f>
@@ -1920,194 +1924,194 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
+          <t>фанера жилых + ГВЛВ с/у</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="inlineStr"/>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>листы вразбежку, не крутить в трубу</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Ламинат 33 кл. / SPC для тёплого пола</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="D40" s="8">
+        <f>Полы!G5+Полы!G6+Полы!G7+Полы!G8</f>
+        <v/>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F40" s="10">
+        <f>IF(D40="","",D40*E40)</f>
+        <v/>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>вкладка Полы, с запасом</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>8–10 мм, допуск на ТП</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>класть на фанеру 12 мм, не на пластины</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Подложка под ламинат для ТП (тонкая 1–2 мм)</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="D41" s="13">
+        <f>Полы!G5+Полы!G6+Полы!G7+Полы!G8</f>
+        <v/>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="F41" s="15">
+        <f>IF(D41="","",D41*E41)</f>
+        <v/>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>вкладка Полы</t>
+        </is>
+      </c>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>не фольгированная толстая</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>не режет тепло</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Пороги / стык ламинат–плитка</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>650</v>
+      </c>
+      <c r="F42" s="10">
+        <f>IF(D42="","",D42*E42)</f>
+        <v/>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
           <t>с/у и вход</t>
         </is>
       </c>
-      <c r="H39" s="12" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr">
         <is>
           <t>алюминий / Т-профиль</t>
         </is>
       </c>
-      <c r="I39" s="12" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="n"/>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="I42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="n"/>
+      <c r="B43" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C40" s="16" t="n"/>
-      <c r="D40" s="16" t="n"/>
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="17">
-        <f>SUM(F36:F39)</f>
-        <v/>
-      </c>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="16" t="n"/>
-      <c r="I40" s="16" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="C43" s="16" t="n"/>
+      <c r="D43" s="16" t="n"/>
+      <c r="E43" s="16" t="n"/>
+      <c r="F43" s="17">
+        <f>SUM(F35:F42)</f>
+        <v/>
+      </c>
+      <c r="G43" s="16" t="n"/>
+      <c r="H43" s="16" t="n"/>
+      <c r="I43" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>5.  Санузел — гидроизоляция, плитка, потолок (МДФ нет)</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="5" t="n"/>
-      <c r="D42" s="5" t="n"/>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>Гидроизоляция обмазочная + лента углов</t>
-        </is>
-      </c>
-      <c r="C43" s="11" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="14" t="n">
-        <v>4200</v>
-      </c>
-      <c r="F43" s="15">
-        <f>IF(D43="","",D43*E43)</f>
-        <v/>
-      </c>
-      <c r="G43" s="12" t="inlineStr">
-        <is>
-          <t>вкладка С_у</t>
-        </is>
-      </c>
-      <c r="H43" s="12" t="inlineStr">
-        <is>
-          <t>Ceresit CR / Knauf Флэхендихт</t>
-        </is>
-      </c>
-      <c r="I43" s="12" t="inlineStr">
-        <is>
-          <t>пол + стены на 2 м</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
-      </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Плитка настенная</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>м²</t>
-        </is>
-      </c>
-      <c r="D44" s="8">
-        <f>'С_у'!D5</f>
-        <v/>
-      </c>
-      <c r="E44" s="9" t="n">
-        <v>1450</v>
-      </c>
-      <c r="F44" s="10">
-        <f>IF(D44="","",D44*E44)</f>
-        <v/>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>вкладка С_у +12%</t>
-        </is>
-      </c>
-      <c r="H44" s="7" t="inlineStr">
-        <is>
-          <t>кафель 250×400 / 200×600</t>
-        </is>
-      </c>
-      <c r="I44" s="7" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>Керамогранит пола с/у</t>
-        </is>
-      </c>
-      <c r="C45" s="11" t="inlineStr">
-        <is>
-          <t>м²</t>
-        </is>
-      </c>
-      <c r="D45" s="13">
-        <f>'С_у'!D6</f>
-        <v/>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>1690</v>
-      </c>
-      <c r="F45" s="15">
-        <f>IF(D45="","",D45*E45)</f>
-        <v/>
-      </c>
-      <c r="G45" s="12" t="inlineStr">
-        <is>
-          <t>вкладка С_у +12%</t>
-        </is>
-      </c>
-      <c r="H45" s="12" t="inlineStr">
-        <is>
-          <t>противоскользящий</t>
-        </is>
-      </c>
-      <c r="I45" s="12" t="inlineStr">
-        <is>
-          <t>поверх ТП</t>
-        </is>
-      </c>
+      <c r="B45" s="5" t="n"/>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="5" t="n"/>
+      <c r="I45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Клей плиточный эластичный C2 S1 (на ТП)</t>
+          <t>Гидроизоляция обмазочная + лента углов</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>кг</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D46" s="8" t="n">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="E46" s="9" t="n">
-        <v>42</v>
+        <v>4200</v>
       </c>
       <c r="F46" s="10">
         <f>IF(D46="","",D46*E46)</f>
@@ -2115,46 +2119,55 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>стены+пол с/у</t>
+          <t>вкладка С_у</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>мешок 25 кг ×3</t>
-        </is>
-      </c>
-      <c r="I46" s="7" t="inlineStr"/>
+          <t>Ceresit CR / Knauf Флэхендихт</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>пол + стены на 2 м</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>Затирка + герметик санитарный</t>
+          <t>Плитка настенная</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="n">
-        <v>1</v>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="D47" s="13">
+        <f>'С_у'!D5</f>
+        <v/>
       </c>
       <c r="E47" s="14" t="n">
-        <v>1800</v>
+        <v>1450</v>
       </c>
       <c r="F47" s="15">
         <f>IF(D47="","",D47*E47)</f>
         <v/>
       </c>
-      <c r="G47" s="12" t="inlineStr"/>
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>вкладка С_у +12%</t>
+        </is>
+      </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>2 кг затирки + 2 тубы</t>
+          <t>кафель 250×400 / 200×600</t>
         </is>
       </c>
       <c r="I47" s="12" t="inlineStr"/>
@@ -2162,66 +2175,80 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>Уголки / раскладка плитки, крестики, клинья</t>
+          <t>Керамогранит пола с/у</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>1</v>
+          <t>м²</t>
+        </is>
+      </c>
+      <c r="D48" s="8">
+        <f>'С_у'!D6</f>
+        <v/>
       </c>
       <c r="E48" s="9" t="n">
-        <v>1200</v>
+        <v>1690</v>
       </c>
       <c r="F48" s="10">
         <f>IF(D48="","",D48*E48)</f>
         <v/>
       </c>
-      <c r="G48" s="7" t="inlineStr"/>
-      <c r="H48" s="7" t="inlineStr"/>
-      <c r="I48" s="7" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>вкладка С_у +12%</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>противоскользящий</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>поверх ТП</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Краска влагостойкая на потолок с/у</t>
+          <t>Клей плиточный эластичный C2 S1 (на ТП)</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>л</t>
+          <t>кг</t>
         </is>
       </c>
       <c r="D49" s="13" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="E49" s="14" t="n">
-        <v>780</v>
+        <v>42</v>
       </c>
       <c r="F49" s="15">
         <f>IF(D49="","",D49*E49)</f>
         <v/>
       </c>
-      <c r="G49" s="12">
-        <f>'С_у'!D7</f>
-        <v/>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>стены+пол с/у</t>
+        </is>
       </c>
       <c r="H49" s="12" t="inlineStr">
         <is>
-          <t>2 слоя</t>
+          <t>мешок 25 кг ×3</t>
         </is>
       </c>
       <c r="I49" s="12" t="inlineStr"/>
@@ -2229,24 +2256,24 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Ревизионный люк / лючок</t>
+          <t>Затирка + герметик санитарный</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D50" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E50" s="9" t="n">
-        <v>1900</v>
+        <v>1800</v>
       </c>
       <c r="F50" s="10">
         <f>IF(D50="","",D50*E50)</f>
@@ -2255,159 +2282,158 @@
       <c r="G50" s="7" t="inlineStr"/>
       <c r="H50" s="7" t="inlineStr">
         <is>
+          <t>2 кг затирки + 2 тубы</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>Уголки / раскладка плитки, крестики, клинья</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="14" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F51" s="15">
+        <f>IF(D51="","",D51*E51)</f>
+        <v/>
+      </c>
+      <c r="G51" s="12" t="inlineStr"/>
+      <c r="H51" s="12" t="inlineStr"/>
+      <c r="I51" s="12" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Краска влагостойкая на потолок с/у</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>л</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>780</v>
+      </c>
+      <c r="F52" s="10">
+        <f>IF(D52="","",D52*E52)</f>
+        <v/>
+      </c>
+      <c r="G52" s="7">
+        <f>'С_у'!D7</f>
+        <v/>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>2 слоя</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>Ревизионный люк / лючок</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="14" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F53" s="15">
+        <f>IF(D53="","",D53*E53)</f>
+        <v/>
+      </c>
+      <c r="G53" s="12" t="inlineStr"/>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
           <t>200×200 / 300×300</t>
         </is>
       </c>
-      <c r="I50" s="7" t="inlineStr">
+      <c r="I53" s="12" t="inlineStr">
         <is>
           <t>если спрятан коллектор/фильтры</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="16" t="n"/>
-      <c r="B51" s="16" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="16" t="n"/>
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C51" s="16" t="n"/>
-      <c r="D51" s="16" t="n"/>
-      <c r="E51" s="16" t="n"/>
-      <c r="F51" s="17">
-        <f>SUM(F43:F50)</f>
-        <v/>
-      </c>
-      <c r="G51" s="16" t="n"/>
-      <c r="H51" s="16" t="n"/>
-      <c r="I51" s="16" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="C54" s="16" t="n"/>
+      <c r="D54" s="16" t="n"/>
+      <c r="E54" s="16" t="n"/>
+      <c r="F54" s="17">
+        <f>SUM(F46:F53)</f>
+        <v/>
+      </c>
+      <c r="G54" s="16" t="n"/>
+      <c r="H54" s="16" t="n"/>
+      <c r="I54" s="16" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>6.  Сантехника — приборы (трубы в разделе 8)</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n"/>
-      <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="5" t="n"/>
-      <c r="I53" s="5" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>6.1</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Унитаз-компакт с сиденьем микролифт</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="9" t="n">
-        <v>8900</v>
-      </c>
-      <c r="F54" s="10">
-        <f>IF(D54="","",D54*E54)</f>
-        <v/>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>план с/у</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr"/>
-      <c r="I54" s="7" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>6.2</t>
-        </is>
-      </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>Душевой поддон 900×900 + ограждение / шторка</t>
-        </is>
-      </c>
-      <c r="C55" s="11" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D55" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="14" t="n">
-        <v>18900</v>
-      </c>
-      <c r="F55" s="15">
-        <f>IF(D55="","",D55*E55)</f>
-        <v/>
-      </c>
-      <c r="G55" s="12" t="inlineStr">
-        <is>
-          <t>душ 0.9×0.9 по плану</t>
-        </is>
-      </c>
-      <c r="H55" s="12" t="inlineStr">
-        <is>
-          <t>акрил + стекло/шторка</t>
-        </is>
-      </c>
-      <c r="I55" s="12" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="inlineStr">
-        <is>
-          <t>6.3</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Смеситель душ с лейкой / стойкой</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D56" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="9" t="n">
-        <v>6200</v>
-      </c>
-      <c r="F56" s="10">
-        <f>IF(D56="","",D56*E56)</f>
-        <v/>
-      </c>
-      <c r="G56" s="7" t="inlineStr"/>
-      <c r="H56" s="7" t="inlineStr"/>
-      <c r="I56" s="7" t="inlineStr"/>
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="5" t="n"/>
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="5" t="n"/>
+      <c r="I56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>Трап душевой / сифон поддона</t>
+          <t>Унитаз-компакт с сиденьем микролифт</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
@@ -2419,25 +2445,29 @@
         <v>1</v>
       </c>
       <c r="E57" s="14" t="n">
-        <v>2400</v>
+        <v>8900</v>
       </c>
       <c r="F57" s="15">
         <f>IF(D57="","",D57*E57)</f>
         <v/>
       </c>
-      <c r="G57" s="12" t="inlineStr"/>
+      <c r="G57" s="12" t="inlineStr">
+        <is>
+          <t>план с/у</t>
+        </is>
+      </c>
       <c r="H57" s="12" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Раковина + сифон + смеситель</t>
+          <t>Душевой поддон 900×900 + ограждение / шторка</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -2449,7 +2479,7 @@
         <v>1</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>7800</v>
+        <v>18900</v>
       </c>
       <c r="F58" s="10">
         <f>IF(D58="","",D58*E58)</f>
@@ -2457,21 +2487,25 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>план с/у</t>
-        </is>
-      </c>
-      <c r="H58" s="7" t="inlineStr"/>
+          <t>душ 0.9×0.9 по плану</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>акрил + стекло/шторка</t>
+        </is>
+      </c>
       <c r="I58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>Полотенцесушитель водяной или электрический</t>
+          <t>Смеситель душ с лейкой / стойкой</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
@@ -2483,67 +2517,55 @@
         <v>1</v>
       </c>
       <c r="E59" s="14" t="n">
-        <v>6500</v>
+        <v>6200</v>
       </c>
       <c r="F59" s="15">
         <f>IF(D59="","",D59*E59)</f>
         <v/>
       </c>
       <c r="G59" s="12" t="inlineStr"/>
-      <c r="H59" s="12" t="inlineStr">
-        <is>
-          <t>электрический проще на сухом ТП</t>
-        </is>
-      </c>
+      <c r="H59" s="12" t="inlineStr"/>
       <c r="I59" s="12" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Смеситель кухня + сифон мойки</t>
+          <t>Трап душевой / сифон поддона</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D60" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>5400</v>
+        <v>2400</v>
       </c>
       <c r="F60" s="10">
         <f>IF(D60="","",D60*E60)</f>
         <v/>
       </c>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>кухня по плану</t>
-        </is>
-      </c>
-      <c r="H60" s="7" t="inlineStr">
-        <is>
-          <t>мойка — в разделе кухня</t>
-        </is>
-      </c>
+      <c r="G60" s="7" t="inlineStr"/>
+      <c r="H60" s="7" t="inlineStr"/>
       <c r="I60" s="7" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t>Фильтр механический + кран шаровый комплект</t>
+          <t>Раковина + сифон + смеситель</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
@@ -2555,7 +2577,7 @@
         <v>1</v>
       </c>
       <c r="E61" s="14" t="n">
-        <v>2800</v>
+        <v>7800</v>
       </c>
       <c r="F61" s="15">
         <f>IF(D61="","",D61*E61)</f>
@@ -2563,180 +2585,176 @@
       </c>
       <c r="G61" s="12" t="inlineStr">
         <is>
-          <t>ввод воды</t>
+          <t>план с/у</t>
         </is>
       </c>
       <c r="H61" s="12" t="inlineStr"/>
       <c r="I61" s="12" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="16" t="n"/>
-      <c r="B62" s="16" t="inlineStr">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>6.6</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Полотенцесушитель водяной или электрический</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F62" s="10">
+        <f>IF(D62="","",D62*E62)</f>
+        <v/>
+      </c>
+      <c r="G62" s="7" t="inlineStr"/>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>электрический проще на сухом ТП</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>Фильтр механический + кран шаровый комплект</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="14" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F63" s="15">
+        <f>IF(D63="","",D63*E63)</f>
+        <v/>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>ввод воды</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="inlineStr"/>
+      <c r="I63" s="12" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="n"/>
+      <c r="B64" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C62" s="16" t="n"/>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="17">
-        <f>SUM(F54:F61)</f>
-        <v/>
-      </c>
-      <c r="G62" s="16" t="n"/>
-      <c r="H62" s="16" t="n"/>
-      <c r="I62" s="16" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="C64" s="16" t="n"/>
+      <c r="D64" s="16" t="n"/>
+      <c r="E64" s="16" t="n"/>
+      <c r="F64" s="17">
+        <f>SUM(F57:F63)</f>
+        <v/>
+      </c>
+      <c r="G64" s="16" t="n"/>
+      <c r="H64" s="16" t="n"/>
+      <c r="I64" s="16" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>7.  Источник тепла (дом без радиаторов, только ТП)</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n"/>
-      <c r="C64" s="5" t="n"/>
-      <c r="D64" s="5" t="n"/>
-      <c r="E64" s="5" t="n"/>
-      <c r="F64" s="5" t="n"/>
-      <c r="G64" s="5" t="n"/>
-      <c r="H64" s="5" t="n"/>
-      <c r="I64" s="5" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>Электрокотёл 6–8 кВт с насосом</t>
-        </is>
-      </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D65" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="14" t="n">
-        <v>28900</v>
-      </c>
-      <c r="F65" s="15">
-        <f>IF(D65="","",D65*E65)</f>
-        <v/>
-      </c>
-      <c r="G65" s="12" t="inlineStr">
-        <is>
-          <t>теплопотери утеплённого барнхауса ~3–5 кВт</t>
-        </is>
-      </c>
-      <c r="H65" s="12" t="inlineStr">
-        <is>
-          <t>Protherm / Эван / Vaillant</t>
-        </is>
-      </c>
-      <c r="I65" s="12" t="inlineStr">
-        <is>
-          <t>можно заменить на тепловой насос — тогда эта строка 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="B66" s="7" t="inlineStr">
-        <is>
-          <t>Бойлер / водонагреватель 80 л</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D66" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="9" t="n">
-        <v>16500</v>
-      </c>
-      <c r="F66" s="10">
-        <f>IF(D66="","",D66*E66)</f>
-        <v/>
-      </c>
-      <c r="G66" s="7" t="inlineStr">
-        <is>
-          <t>ГВС на 2 чел. + запас</t>
-        </is>
-      </c>
-      <c r="H66" s="7" t="inlineStr">
-        <is>
-          <t>накопительный</t>
-        </is>
-      </c>
-      <c r="I66" s="7" t="inlineStr">
-        <is>
-          <t>если котёл двухконтурный — строку обнулить</t>
-        </is>
-      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+      <c r="H66" s="5" t="n"/>
+      <c r="I66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>Группа безопасности + расширительный бак 8–12 л</t>
+          <t>Электрокотёл 6–8 кВт с насосом</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D67" s="13" t="n">
         <v>1</v>
       </c>
       <c r="E67" s="14" t="n">
-        <v>5400</v>
+        <v>28900</v>
       </c>
       <c r="F67" s="15">
         <f>IF(D67="","",D67*E67)</f>
         <v/>
       </c>
-      <c r="G67" s="12" t="inlineStr"/>
-      <c r="H67" s="12" t="inlineStr"/>
-      <c r="I67" s="12" t="inlineStr"/>
+      <c r="G67" s="12" t="inlineStr">
+        <is>
+          <t>теплопотери утеплённого барнхауса ~3–5 кВт</t>
+        </is>
+      </c>
+      <c r="H67" s="12" t="inlineStr">
+        <is>
+          <t>Protherm / Эван / Vaillant</t>
+        </is>
+      </c>
+      <c r="I67" s="12" t="inlineStr">
+        <is>
+          <t>можно заменить на тепловой насос — тогда эта строка 0</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Труба подачи котёл–коллектор PEX/PP 25 мм + изоляция</t>
+          <t>Бойлер / водонагреватель 80 л</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>м</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D68" s="8" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E68" s="9" t="n">
-        <v>145</v>
+        <v>16500</v>
       </c>
       <c r="F68" s="10">
         <f>IF(D68="","",D68*E68)</f>
@@ -2744,21 +2762,29 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>котельная/кухня → коллектор</t>
-        </is>
-      </c>
-      <c r="H68" s="7" t="inlineStr"/>
-      <c r="I68" s="7" t="inlineStr"/>
+          <t>ГВС на 2 чел. + запас</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>накопительный</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>если котёл двухконтурный — строку обнулить</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>Краны, грязевик, термоманометр</t>
+          <t>Группа безопасности + расширительный бак 8–12 л</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
@@ -2770,7 +2796,7 @@
         <v>1</v>
       </c>
       <c r="E69" s="14" t="n">
-        <v>3200</v>
+        <v>5400</v>
       </c>
       <c r="F69" s="15">
         <f>IF(D69="","",D69*E69)</f>
@@ -2781,119 +2807,111 @@
       <c r="I69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="16" t="n"/>
-      <c r="B70" s="16" t="inlineStr">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Труба подачи котёл–коллектор PEX/PP 25 мм + изоляция</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>145</v>
+      </c>
+      <c r="F70" s="10">
+        <f>IF(D70="","",D70*E70)</f>
+        <v/>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>котельная → коллектор</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr"/>
+      <c r="I70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>Краны, грязевик, термоманометр</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="14" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F71" s="15">
+        <f>IF(D71="","",D71*E71)</f>
+        <v/>
+      </c>
+      <c r="G71" s="12" t="inlineStr"/>
+      <c r="H71" s="12" t="inlineStr"/>
+      <c r="I71" s="12" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="n"/>
+      <c r="B72" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C70" s="16" t="n"/>
-      <c r="D70" s="16" t="n"/>
-      <c r="E70" s="16" t="n"/>
-      <c r="F70" s="17">
-        <f>SUM(F65:F69)</f>
-        <v/>
-      </c>
-      <c r="G70" s="16" t="n"/>
-      <c r="H70" s="16" t="n"/>
-      <c r="I70" s="16" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
+      <c r="C72" s="16" t="n"/>
+      <c r="D72" s="16" t="n"/>
+      <c r="E72" s="16" t="n"/>
+      <c r="F72" s="17">
+        <f>SUM(F67:F71)</f>
+        <v/>
+      </c>
+      <c r="G72" s="16" t="n"/>
+      <c r="H72" s="16" t="n"/>
+      <c r="I72" s="16" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>8.  Водопровод и канализация внутри дома</t>
         </is>
       </c>
-      <c r="B72" s="5" t="n"/>
-      <c r="C72" s="5" t="n"/>
-      <c r="D72" s="5" t="n"/>
-      <c r="E72" s="5" t="n"/>
-      <c r="F72" s="5" t="n"/>
-      <c r="G72" s="5" t="n"/>
-      <c r="H72" s="5" t="n"/>
-      <c r="I72" s="5" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="11" t="inlineStr">
-        <is>
-          <t>8.1</t>
-        </is>
-      </c>
-      <c r="B73" s="12" t="inlineStr">
-        <is>
-          <t>Труба PPR / PEX 20 мм холод+горяч</t>
-        </is>
-      </c>
-      <c r="C73" s="11" t="inlineStr">
-        <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="D73" s="13" t="n">
-        <v>36</v>
-      </c>
-      <c r="E73" s="14" t="n">
-        <v>78</v>
-      </c>
-      <c r="F73" s="15">
-        <f>IF(D73="","",D73*E73)</f>
-        <v/>
-      </c>
-      <c r="G73" s="12" t="inlineStr">
-        <is>
-          <t>с/у + кухня + бойлер</t>
-        </is>
-      </c>
-      <c r="H73" s="12" t="inlineStr"/>
-      <c r="I73" s="12" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>8.2</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t>Труба канализация 50 мм + отводы</t>
-        </is>
-      </c>
-      <c r="C74" s="6" t="inlineStr">
-        <is>
-          <t>м</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E74" s="9" t="n">
-        <v>165</v>
-      </c>
-      <c r="F74" s="10">
-        <f>IF(D74="","",D74*E74)</f>
-        <v/>
-      </c>
-      <c r="G74" s="7" t="inlineStr">
-        <is>
-          <t>умывальник, душ, стиралка, кухня</t>
-        </is>
-      </c>
-      <c r="H74" s="7" t="inlineStr">
-        <is>
-          <t>серая ПП</t>
-        </is>
-      </c>
-      <c r="I74" s="7" t="inlineStr"/>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="5" t="n"/>
+      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="5" t="n"/>
+      <c r="F74" s="5" t="n"/>
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="5" t="n"/>
+      <c r="I74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>Труба канализация 110 мм + тройники</t>
+          <t>Труба PPR / PEX 20 мм холод+горяч</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
@@ -2902,10 +2920,10 @@
         </is>
       </c>
       <c r="D75" s="13" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E75" s="14" t="n">
-        <v>290</v>
+        <v>78</v>
       </c>
       <c r="F75" s="15">
         <f>IF(D75="","",D75*E75)</f>
@@ -2913,210 +2931,210 @@
       </c>
       <c r="G75" s="12" t="inlineStr">
         <is>
-          <t>унитаз + выпуск</t>
+          <t>с/у + бойлер, без кухни</t>
         </is>
       </c>
       <c r="H75" s="12" t="inlineStr"/>
-      <c r="I75" s="12" t="inlineStr">
-        <is>
-          <t>выпуск до наружной трубы — внутри дома</t>
-        </is>
-      </c>
+      <c r="I75" s="12" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>Клипсы, хомуты, манжеты, ревизия</t>
+          <t>Труба канализация 50 мм + отводы</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>м</t>
         </is>
       </c>
       <c r="D76" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E76" s="9" t="n">
-        <v>2100</v>
+        <v>165</v>
       </c>
       <c r="F76" s="10">
         <f>IF(D76="","",D76*E76)</f>
         <v/>
       </c>
-      <c r="G76" s="7" t="inlineStr"/>
-      <c r="H76" s="7" t="inlineStr"/>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>умывальник, душ, стиралка</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>серая ПП</t>
+        </is>
+      </c>
       <c r="I76" s="7" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>Гибкие подводки 2 шт × 4 точки</t>
+          <t>Труба канализация 110 мм + тройники</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>м</t>
         </is>
       </c>
       <c r="D77" s="13" t="n">
         <v>8</v>
       </c>
       <c r="E77" s="14" t="n">
-        <v>220</v>
+        <v>290</v>
       </c>
       <c r="F77" s="15">
         <f>IF(D77="","",D77*E77)</f>
         <v/>
       </c>
-      <c r="G77" s="12" t="inlineStr"/>
-      <c r="H77" s="12" t="inlineStr">
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>унитаз + выпуск</t>
+        </is>
+      </c>
+      <c r="H77" s="12" t="inlineStr"/>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>выпуск до наружной трубы — внутри дома</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>8.4</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Клипсы, хомуты, манжеты, ревизия</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F78" s="10">
+        <f>IF(D78="","",D78*E78)</f>
+        <v/>
+      </c>
+      <c r="G78" s="7" t="inlineStr"/>
+      <c r="H78" s="7" t="inlineStr"/>
+      <c r="I78" s="7" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>Гибкие подводки</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E79" s="14" t="n">
+        <v>220</v>
+      </c>
+      <c r="F79" s="15">
+        <f>IF(D79="","",D79*E79)</f>
+        <v/>
+      </c>
+      <c r="G79" s="12" t="inlineStr">
+        <is>
+          <t>с/у точки</t>
+        </is>
+      </c>
+      <c r="H79" s="12" t="inlineStr">
         <is>
           <t>40–50 см</t>
         </is>
       </c>
-      <c r="I77" s="12" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="16" t="n"/>
-      <c r="B78" s="16" t="inlineStr">
+      <c r="I79" s="12" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="n"/>
+      <c r="B80" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C78" s="16" t="n"/>
-      <c r="D78" s="16" t="n"/>
-      <c r="E78" s="16" t="n"/>
-      <c r="F78" s="17">
-        <f>SUM(F73:F77)</f>
-        <v/>
-      </c>
-      <c r="G78" s="16" t="n"/>
-      <c r="H78" s="16" t="n"/>
-      <c r="I78" s="16" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+      <c r="C80" s="16" t="n"/>
+      <c r="D80" s="16" t="n"/>
+      <c r="E80" s="16" t="n"/>
+      <c r="F80" s="17">
+        <f>SUM(F75:F79)</f>
+        <v/>
+      </c>
+      <c r="G80" s="16" t="n"/>
+      <c r="H80" s="16" t="n"/>
+      <c r="I80" s="16" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>9.  Электрика</t>
         </is>
       </c>
-      <c r="B80" s="5" t="n"/>
-      <c r="C80" s="5" t="n"/>
-      <c r="D80" s="5" t="n"/>
-      <c r="E80" s="5" t="n"/>
-      <c r="F80" s="5" t="n"/>
-      <c r="G80" s="5" t="n"/>
-      <c r="H80" s="5" t="n"/>
-      <c r="I80" s="5" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="11" t="inlineStr">
-        <is>
-          <t>9.1</t>
-        </is>
-      </c>
-      <c r="B81" s="12" t="inlineStr">
-        <is>
-          <t>Щиток навесной 18 модулей + DIN</t>
-        </is>
-      </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D81" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E81" s="14" t="n">
-        <v>3200</v>
-      </c>
-      <c r="F81" s="15">
-        <f>IF(D81="","",D81*E81)</f>
-        <v/>
-      </c>
-      <c r="G81" s="12" t="inlineStr">
-        <is>
-          <t>холл / кухня</t>
-        </is>
-      </c>
-      <c r="H81" s="12" t="inlineStr"/>
-      <c r="I81" s="12" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>9.2</t>
-        </is>
-      </c>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>Автоматы, УЗО, реле напряжения, нулевые шины</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D82" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E82" s="9" t="n">
-        <v>9800</v>
-      </c>
-      <c r="F82" s="10">
-        <f>IF(D82="","",D82*E82)</f>
-        <v/>
-      </c>
-      <c r="G82" s="7" t="inlineStr">
-        <is>
-          <t>свет, розетки, плита, стиралка, котёл, бойлер</t>
-        </is>
-      </c>
-      <c r="H82" s="7" t="inlineStr">
-        <is>
-          <t>ABB / IEK / Systeme</t>
-        </is>
-      </c>
-      <c r="I82" s="7" t="inlineStr">
-        <is>
-          <t>отдельные линии на мокрые и 3 кВт+</t>
-        </is>
-      </c>
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="5" t="n"/>
+      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="5" t="n"/>
+      <c r="F82" s="5" t="n"/>
+      <c r="G82" s="5" t="n"/>
+      <c r="H82" s="5" t="n"/>
+      <c r="I82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="11" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B83" s="12" t="inlineStr">
         <is>
-          <t>Кабель ВВГнг-LS 3×2.5</t>
+          <t>Щиток навесной 18 модулей + DIN</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>м</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D83" s="13" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="E83" s="14" t="n">
-        <v>86</v>
+        <v>3200</v>
       </c>
       <c r="F83" s="15">
         <f>IF(D83="","",D83*E83)</f>
@@ -3124,7 +3142,7 @@
       </c>
       <c r="G83" s="12" t="inlineStr">
         <is>
-          <t>розетки</t>
+          <t>холл</t>
         </is>
       </c>
       <c r="H83" s="12" t="inlineStr"/>
@@ -3133,24 +3151,24 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>Кабель ВВГнг-LS 3×1.5</t>
+          <t>Автоматы, УЗО, реле напряжения, нулевые шины</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>м</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D84" s="8" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>58</v>
+        <v>8900</v>
       </c>
       <c r="F84" s="10">
         <f>IF(D84="","",D84*E84)</f>
@@ -3158,21 +3176,29 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>освещение</t>
-        </is>
-      </c>
-      <c r="H84" s="7" t="inlineStr"/>
-      <c r="I84" s="7" t="inlineStr"/>
+          <t>свет, розетки, стиралка, котёл, бойлер</t>
+        </is>
+      </c>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>ABB / IEK / Systeme</t>
+        </is>
+      </c>
+      <c r="I84" s="7" t="inlineStr">
+        <is>
+          <t>без линии плиты — кухню не закладываем</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="11" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t>Кабель ВВГнг-LS 3×4 (плита / котёл)</t>
+          <t>Кабель ВВГнг-LS 3×2.5</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
@@ -3181,10 +3207,10 @@
         </is>
       </c>
       <c r="D85" s="13" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="E85" s="14" t="n">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="F85" s="15">
         <f>IF(D85="","",D85*E85)</f>
@@ -3192,7 +3218,7 @@
       </c>
       <c r="G85" s="12" t="inlineStr">
         <is>
-          <t>2 линии</t>
+          <t>розетки</t>
         </is>
       </c>
       <c r="H85" s="12" t="inlineStr"/>
@@ -3201,12 +3227,12 @@
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>9.6</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Гофра ПВХ 16–20 мм + клипсы</t>
+          <t>Кабель ВВГнг-LS 3×1.5</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -3215,10 +3241,10 @@
         </is>
       </c>
       <c r="D86" s="8" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="E86" s="9" t="n">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="F86" s="10">
         <f>IF(D86="","",D86*E86)</f>
@@ -3226,67 +3252,67 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>по каркасу</t>
+          <t>освещение</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr"/>
-      <c r="I86" s="7" t="inlineStr">
-        <is>
-          <t>перегородки уже стоят — тянем в пустотах</t>
-        </is>
-      </c>
+      <c r="I86" s="7" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="11" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>Подрозетники</t>
+          <t>Кабель ВВГнг-LS 3×4 (котёл / бойлер)</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>м</t>
         </is>
       </c>
       <c r="D87" s="13" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E87" s="14" t="n">
-        <v>28</v>
+        <v>128</v>
       </c>
       <c r="F87" s="15">
         <f>IF(D87="","",D87*E87)</f>
         <v/>
       </c>
-      <c r="G87" s="12" t="inlineStr"/>
+      <c r="G87" s="12" t="inlineStr">
+        <is>
+          <t>1 линия</t>
+        </is>
+      </c>
       <c r="H87" s="12" t="inlineStr"/>
       <c r="I87" s="12" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>Розетки 16А</t>
+          <t>Гофра ПВХ 16–20 мм + клипсы</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>м</t>
         </is>
       </c>
       <c r="D88" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="E88" s="9" t="n">
         <v>22</v>
-      </c>
-      <c r="E88" s="9" t="n">
-        <v>240</v>
       </c>
       <c r="F88" s="10">
         <f>IF(D88="","",D88*E88)</f>
@@ -3294,25 +3320,25 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>по комнатам + кухня + с/у IP44</t>
+          <t>по каркасу</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr"/>
       <c r="I88" s="7" t="inlineStr">
         <is>
-          <t>без техники</t>
+          <t>перегородки уже стоят — тянем в пустотах</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="11" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="B89" s="12" t="inlineStr">
         <is>
-          <t>Выключатели / проходные</t>
+          <t>Подрозетники</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
@@ -3321,10 +3347,10 @@
         </is>
       </c>
       <c r="D89" s="13" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="E89" s="14" t="n">
-        <v>260</v>
+        <v>28</v>
       </c>
       <c r="F89" s="15">
         <f>IF(D89="","",D89*E89)</f>
@@ -3337,12 +3363,12 @@
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>9.10</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Светильники потолочные / трек (жилые)</t>
+          <t>Розетки 16А</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -3351,10 +3377,10 @@
         </is>
       </c>
       <c r="D90" s="8" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E90" s="9" t="n">
-        <v>1900</v>
+        <v>240</v>
       </c>
       <c r="F90" s="10">
         <f>IF(D90="","",D90*E90)</f>
@@ -3362,25 +3388,25 @@
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>скатный потолок — накладные / шина</t>
+          <t>по комнатам + с/у IP44</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr"/>
       <c r="I90" s="7" t="inlineStr">
         <is>
-          <t>можно заменить своими</t>
+          <t>без кухонного блока</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="11" t="inlineStr">
         <is>
-          <t>9.11</t>
+          <t>9.9</t>
         </is>
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
-          <t>Светильник с/у IP44 + подсветка зеркала</t>
+          <t>Выключатели / проходные</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
@@ -3389,10 +3415,10 @@
         </is>
       </c>
       <c r="D91" s="13" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E91" s="14" t="n">
-        <v>1600</v>
+        <v>260</v>
       </c>
       <c r="F91" s="15">
         <f>IF(D91="","",D91*E91)</f>
@@ -3405,12 +3431,12 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>9.12</t>
+          <t>9.10</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Вентилятор с/у Ø100 с обратным клапаном</t>
+          <t>Светильники потолочные / трек (жилые)</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -3419,10 +3445,10 @@
         </is>
       </c>
       <c r="D92" s="8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E92" s="9" t="n">
-        <v>2100</v>
+        <v>1900</v>
       </c>
       <c r="F92" s="10">
         <f>IF(D92="","",D92*E92)</f>
@@ -3430,37 +3456,37 @@
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>в стену / через кровлю</t>
-        </is>
-      </c>
-      <c r="H92" s="7" t="inlineStr">
-        <is>
-          <t>вытяжка</t>
-        </is>
-      </c>
-      <c r="I92" s="7" t="inlineStr"/>
+          <t>скатный потолок — накладные / шина</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr"/>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t>можно заменить своими</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="11" t="inlineStr">
         <is>
-          <t>9.13</t>
+          <t>9.11</t>
         </is>
       </c>
       <c r="B93" s="12" t="inlineStr">
         <is>
-          <t>Воздуховод 100 мм + решётка + герметик</t>
+          <t>Светильник с/у IP44 + подсветка зеркала</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D93" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E93" s="14" t="n">
-        <v>1400</v>
+        <v>1600</v>
       </c>
       <c r="F93" s="15">
         <f>IF(D93="","",D93*E93)</f>
@@ -3473,147 +3499,143 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>9.14</t>
+          <t>9.12</t>
         </is>
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>Клеммы WAGO, изолента, маркировка</t>
+          <t>Вентилятор с/у Ø100 с обратным клапаном</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>компл</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D94" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E94" s="9" t="n">
-        <v>1800</v>
+        <v>2100</v>
       </c>
       <c r="F94" s="10">
         <f>IF(D94="","",D94*E94)</f>
         <v/>
       </c>
-      <c r="G94" s="7" t="inlineStr"/>
-      <c r="H94" s="7" t="inlineStr"/>
+      <c r="G94" s="7" t="inlineStr">
+        <is>
+          <t>в стену / через кровлю</t>
+        </is>
+      </c>
+      <c r="H94" s="7" t="inlineStr">
+        <is>
+          <t>вытяжка</t>
+        </is>
+      </c>
       <c r="I94" s="7" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="16" t="n"/>
-      <c r="B95" s="16" t="inlineStr">
+      <c r="A95" s="11" t="inlineStr">
+        <is>
+          <t>9.13</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>Воздуховод 100 мм + решётка + герметик</t>
+        </is>
+      </c>
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D95" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="14" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F95" s="15">
+        <f>IF(D95="","",D95*E95)</f>
+        <v/>
+      </c>
+      <c r="G95" s="12" t="inlineStr"/>
+      <c r="H95" s="12" t="inlineStr"/>
+      <c r="I95" s="12" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="inlineStr">
+        <is>
+          <t>9.14</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>Клеммы WAGO, изолента, маркировка</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="9" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F96" s="10">
+        <f>IF(D96="","",D96*E96)</f>
+        <v/>
+      </c>
+      <c r="G96" s="7" t="inlineStr"/>
+      <c r="H96" s="7" t="inlineStr"/>
+      <c r="I96" s="7" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="n"/>
+      <c r="B97" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C95" s="16" t="n"/>
-      <c r="D95" s="16" t="n"/>
-      <c r="E95" s="16" t="n"/>
-      <c r="F95" s="17">
-        <f>SUM(F81:F94)</f>
-        <v/>
-      </c>
-      <c r="G95" s="16" t="n"/>
-      <c r="H95" s="16" t="n"/>
-      <c r="I95" s="16" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="4" t="inlineStr">
-        <is>
-          <t>10.  Кухня — встроенные материалы (гарнитур целиком можно заменить одной строкой)</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="n"/>
-      <c r="C97" s="5" t="n"/>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="5" t="n"/>
-      <c r="F97" s="5" t="n"/>
-      <c r="G97" s="5" t="n"/>
-      <c r="H97" s="5" t="n"/>
-      <c r="I97" s="5" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="6" t="inlineStr">
-        <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>Мойка врезная нерж. 600 мм</t>
-        </is>
-      </c>
-      <c r="C98" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D98" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E98" s="9" t="n">
-        <v>4200</v>
-      </c>
-      <c r="F98" s="10">
-        <f>IF(D98="","",D98*E98)</f>
-        <v/>
-      </c>
-      <c r="G98" s="7" t="inlineStr">
-        <is>
-          <t>план кухни</t>
-        </is>
-      </c>
-      <c r="H98" s="7" t="inlineStr"/>
-      <c r="I98" s="7" t="inlineStr"/>
+      <c r="C97" s="16" t="n"/>
+      <c r="D97" s="16" t="n"/>
+      <c r="E97" s="16" t="n"/>
+      <c r="F97" s="17">
+        <f>SUM(F83:F96)</f>
+        <v/>
+      </c>
+      <c r="G97" s="16" t="n"/>
+      <c r="H97" s="16" t="n"/>
+      <c r="I97" s="16" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="11" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="B99" s="12" t="inlineStr">
-        <is>
-          <t>Столешница 38 мм, 2.4 м + пристенный бортик</t>
-        </is>
-      </c>
-      <c r="C99" s="11" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D99" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E99" s="14" t="n">
-        <v>9800</v>
-      </c>
-      <c r="F99" s="15">
-        <f>IF(D99="","",D99*E99)</f>
-        <v/>
-      </c>
-      <c r="G99" s="12" t="inlineStr">
-        <is>
-          <t>кухня 2.4 м по плану</t>
-        </is>
-      </c>
-      <c r="H99" s="12" t="inlineStr">
-        <is>
-          <t>влагостойкая</t>
-        </is>
-      </c>
-      <c r="I99" s="12" t="inlineStr"/>
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>10.  Прочее и расходники</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="n"/>
+      <c r="C99" s="5" t="n"/>
+      <c r="D99" s="5" t="n"/>
+      <c r="E99" s="5" t="n"/>
+      <c r="F99" s="5" t="n"/>
+      <c r="G99" s="5" t="n"/>
+      <c r="H99" s="5" t="n"/>
+      <c r="I99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>Фартук плитка / панель 2.4×0.6 м</t>
+          <t>Пена, герметик акрил/силикон, клей жидкие гвозди</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
@@ -3625,7 +3647,7 @@
         <v>1</v>
       </c>
       <c r="E100" s="9" t="n">
-        <v>4500</v>
+        <v>2800</v>
       </c>
       <c r="F100" s="10">
         <f>IF(D100="","",D100*E100)</f>
@@ -3633,33 +3655,29 @@
       </c>
       <c r="G100" s="7" t="inlineStr"/>
       <c r="H100" s="7" t="inlineStr"/>
-      <c r="I100" s="7" t="inlineStr">
-        <is>
-          <t>если панель — без клея плитки</t>
-        </is>
-      </c>
+      <c r="I100" s="7" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="11" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B101" s="12" t="inlineStr">
         <is>
-          <t>Варочная панель электрическая 60 см (если нет своей)</t>
+          <t>Грунтовка универсальная + влагостойкая</t>
         </is>
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>л</t>
         </is>
       </c>
       <c r="D101" s="13" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E101" s="14" t="n">
-        <v>14500</v>
+        <v>220</v>
       </c>
       <c r="F101" s="15">
         <f>IF(D101="","",D101*E101)</f>
@@ -3667,37 +3685,33 @@
       </c>
       <c r="G101" s="12" t="inlineStr">
         <is>
-          <t>план: плита</t>
+          <t>ГВЛ, с/у</t>
         </is>
       </c>
       <c r="H101" s="12" t="inlineStr"/>
-      <c r="I101" s="12" t="inlineStr">
-        <is>
-          <t>обнулите, если техника своя</t>
-        </is>
-      </c>
+      <c r="I101" s="12" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>Вытяжка 60 см + воздуховод</t>
+          <t>Плёнка укрывная, скотч малярный, мешки</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>компл</t>
         </is>
       </c>
       <c r="D102" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E102" s="9" t="n">
-        <v>8900</v>
+        <v>1200</v>
       </c>
       <c r="F102" s="10">
         <f>IF(D102="","",D102*E102)</f>
@@ -3707,238 +3721,106 @@
       <c r="H102" s="7" t="inlineStr"/>
       <c r="I102" s="7" t="inlineStr">
         <is>
-          <t>обнулите, если своя</t>
+          <t>для отделки, не строительная пароизоляция</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="16" t="n"/>
-      <c r="B103" s="16" t="inlineStr">
+      <c r="A103" s="11" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>Крепёж смешанный (анкера, уголки, дюбели)</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="D103" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="14" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F103" s="15">
+        <f>IF(D103="","",D103*E103)</f>
+        <v/>
+      </c>
+      <c r="G103" s="12" t="inlineStr"/>
+      <c r="H103" s="12" t="inlineStr"/>
+      <c r="I103" s="12" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="n"/>
+      <c r="B104" s="16" t="inlineStr">
         <is>
           <t>Итого по разделу</t>
         </is>
       </c>
-      <c r="C103" s="16" t="n"/>
-      <c r="D103" s="16" t="n"/>
-      <c r="E103" s="16" t="n"/>
-      <c r="F103" s="17">
-        <f>SUM(F98:F102)</f>
-        <v/>
-      </c>
-      <c r="G103" s="16" t="n"/>
-      <c r="H103" s="16" t="n"/>
-      <c r="I103" s="16" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="inlineStr">
-        <is>
-          <t>11.  Прочее и расходники</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="n"/>
-      <c r="C105" s="5" t="n"/>
-      <c r="D105" s="5" t="n"/>
-      <c r="E105" s="5" t="n"/>
-      <c r="F105" s="5" t="n"/>
-      <c r="G105" s="5" t="n"/>
-      <c r="H105" s="5" t="n"/>
-      <c r="I105" s="5" t="n"/>
+      <c r="C104" s="16" t="n"/>
+      <c r="D104" s="16" t="n"/>
+      <c r="E104" s="16" t="n"/>
+      <c r="F104" s="17">
+        <f>SUM(F100:F103)</f>
+        <v/>
+      </c>
+      <c r="G104" s="16" t="n"/>
+      <c r="H104" s="16" t="n"/>
+      <c r="I104" s="16" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>11.1</t>
-        </is>
-      </c>
-      <c r="B106" s="7" t="inlineStr">
-        <is>
-          <t>Пена, герметик акрил/силикон, клей жидкие гвозди</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D106" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E106" s="9" t="n">
-        <v>2800</v>
-      </c>
-      <c r="F106" s="10">
-        <f>IF(D106="","",D106*E106)</f>
-        <v/>
-      </c>
-      <c r="G106" s="7" t="inlineStr"/>
-      <c r="H106" s="7" t="inlineStr"/>
-      <c r="I106" s="7" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="11" t="inlineStr">
-        <is>
-          <t>11.2</t>
-        </is>
-      </c>
-      <c r="B107" s="12" t="inlineStr">
-        <is>
-          <t>Грунтовка универсальная + влагостойкая</t>
-        </is>
-      </c>
-      <c r="C107" s="11" t="inlineStr">
-        <is>
-          <t>л</t>
-        </is>
-      </c>
-      <c r="D107" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="E107" s="14" t="n">
-        <v>220</v>
-      </c>
-      <c r="F107" s="15">
-        <f>IF(D107="","",D107*E107)</f>
-        <v/>
-      </c>
-      <c r="G107" s="12" t="inlineStr">
-        <is>
-          <t>ГВЛ, с/у</t>
-        </is>
-      </c>
-      <c r="H107" s="12" t="inlineStr"/>
-      <c r="I107" s="12" t="inlineStr"/>
+      <c r="A106" s="18" t="inlineStr">
+        <is>
+          <t>ИТОГО МАТЕРИАЛЫ (без работ, без окон/дверей/террасы/утепления контура)</t>
+        </is>
+      </c>
+      <c r="B106" s="18" t="n"/>
+      <c r="C106" s="18" t="n"/>
+      <c r="D106" s="18" t="n"/>
+      <c r="E106" s="18" t="n"/>
+      <c r="F106" s="19">
+        <f>F10+F21+F32+F43+F54+F64+F72+F80+F97+F104</f>
+        <v/>
+      </c>
+      <c r="G106" s="18" t="n"/>
+      <c r="H106" s="18" t="n"/>
+      <c r="I106" s="18" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>11.3</t>
-        </is>
-      </c>
-      <c r="B108" s="7" t="inlineStr">
-        <is>
-          <t>Плёнка укрывная, скотч малярный, мешки</t>
-        </is>
-      </c>
-      <c r="C108" s="6" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D108" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E108" s="9" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F108" s="10">
-        <f>IF(D108="","",D108*E108)</f>
-        <v/>
-      </c>
-      <c r="G108" s="7" t="inlineStr"/>
-      <c r="H108" s="7" t="inlineStr"/>
-      <c r="I108" s="7" t="inlineStr">
-        <is>
-          <t>для отделки, не строительная пароизоляция</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="11" t="inlineStr">
-        <is>
-          <t>11.4</t>
-        </is>
-      </c>
-      <c r="B109" s="12" t="inlineStr">
-        <is>
-          <t>Крепёж смешанный (анкера, уголки, дюбели)</t>
-        </is>
-      </c>
-      <c r="C109" s="11" t="inlineStr">
-        <is>
-          <t>компл</t>
-        </is>
-      </c>
-      <c r="D109" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E109" s="14" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F109" s="15">
-        <f>IF(D109="","",D109*E109)</f>
-        <v/>
-      </c>
-      <c r="G109" s="12" t="inlineStr"/>
-      <c r="H109" s="12" t="inlineStr"/>
-      <c r="I109" s="12" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="16" t="n"/>
-      <c r="B110" s="16" t="inlineStr">
-        <is>
-          <t>Итого по разделу</t>
-        </is>
-      </c>
-      <c r="C110" s="16" t="n"/>
-      <c r="D110" s="16" t="n"/>
-      <c r="E110" s="16" t="n"/>
-      <c r="F110" s="17">
-        <f>SUM(F106:F109)</f>
-        <v/>
-      </c>
-      <c r="G110" s="16" t="n"/>
-      <c r="H110" s="16" t="n"/>
-      <c r="I110" s="16" t="n"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="18" t="inlineStr">
-        <is>
-          <t>ИТОГО МАТЕРИАЛЫ (без работ, без окон/дверей/террасы/утепления контура)</t>
-        </is>
-      </c>
-      <c r="B112" s="18" t="n"/>
-      <c r="C112" s="18" t="n"/>
-      <c r="D112" s="18" t="n"/>
-      <c r="E112" s="18" t="n"/>
-      <c r="F112" s="19">
-        <f>F11+F22+F33+F40+F51+F62+F70+F78+F95+F103+F110</f>
-        <v/>
-      </c>
-      <c r="G112" s="18" t="n"/>
-      <c r="H112" s="18" t="n"/>
-      <c r="I112" s="18" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="20" t="inlineStr">
-        <is>
-          <t>Как пользоваться: меняйте столбец «Цена, ₽» — сумма раздела и итог пересчитаются. Количество с формулой тянется с вкладок Полы / Стены / Потолки / Обшивка / Теплый_пол / С_у. Строки техники (котёл, бойлер, варочная, вытяжка) обнулите в «Кол-во», если привезёте своё. Работы, окна, двери, утепление и плёнка наружного контура, каркасы перегородок и вся терраса в смету не входят. Цены — ориентир Петрович СПб / Valtec, сентябрь 2026; перед закупкой сверьте карточку товара. Отделка: МДФ дуб альпийский 2600×238×6 (Союз), без лака — покрытие уже на панели. Кухня: гарнитур целиком не заложен, только мойка, столешница, фартук и базовая техника.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
+      <c r="A108" s="20" t="inlineStr">
+        <is>
+          <t>Как пользоваться: меняйте столбец «Цена, ₽» — сумма раздела и итог пересчитаются. Количество с формулой тянется с вкладок Полы / Стены / Потолки / Обшивка / Теплый_пол / С_у. Строки техники (котёл, бойлер) обнулите в «Кол-во», если привезёте своё. Работы, окна, двери, утепление и плёнка наружного контура, каркасы перегородок и вся терраса в смету не входят. Цены — ориентир Петрович СПб / Valtec, сентябрь 2026; перед закупкой сверьте карточку товара. Отделка: МДФ дуб альпийский 2600×238×6 (Союз), без лака — покрытие уже на панели. Кухня (гарнитур, мойка, плита, вытяжка, смеситель) в смету не входит.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
   </sheetData>
-  <autoFilter ref="A4:I112"/>
-  <mergeCells count="15">
-    <mergeCell ref="A64:I64"/>
-    <mergeCell ref="A97:I97"/>
+  <autoFilter ref="A4:I106"/>
+  <mergeCells count="14">
+    <mergeCell ref="A82:I82"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A105:I105"/>
+    <mergeCell ref="A108:I114"/>
+    <mergeCell ref="A99:I99"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A112:E112"/>
+    <mergeCell ref="A66:I66"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A80:I80"/>
-    <mergeCell ref="A53:I53"/>
-    <mergeCell ref="A114:I120"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A72:I72"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A74:I74"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A106:E106"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -4618,7 +4500,7 @@
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>Пластина VT.FP.SZ.0125 = 1000×125 мм, труба Ø16. Пачка 40 шт. Норма 6.4 шт/м² ≈ 80% покрытия (на петлях пластин нет). Контур не длиннее 80–90 м — отсюда число петель. Пол уже утеплён и под плёнкой: подложку под пластины не закладывал.</t>
+          <t>Пластина VT.FP.SZ.0125 = 1000×125 мм, труба Ø16. Пачка 40 шт. Норма 6.4 шт/м² ≈ 80% покрытия (на петлях пластин нет). Контур не длиннее 80–90 м — отсюда число петель. Пол уже утеплён и под плёнкой: подложку под пластины не закладывал. Сверху на пластины — фанера 12 мм (жилые) / ГВЛВ (с/у), затем финиш. Не класть ламинат на пластины.</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5324,15 +5206,15 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>1. Перегородки — заполнение и обшивка</t>
+          <t>1. Перегородки — вата + ГВЛВ с/у</t>
         </is>
       </c>
       <c r="C5" s="14">
-        <f>Смета!F11</f>
+        <f>Смета!F10</f>
         <v/>
       </c>
       <c r="D5" s="22">
-        <f>IF($C$17=0,0,C5/$C$17)</f>
+        <f>IF($C$16=0,0,C5/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5346,11 +5228,11 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>Смета!F22</f>
+        <f>Смета!F21</f>
         <v/>
       </c>
       <c r="D6" s="24">
-        <f>IF($C$17=0,0,C6/$C$17)</f>
+        <f>IF($C$16=0,0,C6/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5364,11 +5246,11 @@
         </is>
       </c>
       <c r="C7" s="14">
-        <f>Смета!F33</f>
+        <f>Смета!F32</f>
         <v/>
       </c>
       <c r="D7" s="22">
-        <f>IF($C$17=0,0,C7/$C$17)</f>
+        <f>IF($C$16=0,0,C7/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5378,15 +5260,15 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>4. Финиш пола</t>
+          <t>4. Настил пола и ламинат</t>
         </is>
       </c>
       <c r="C8" s="9">
-        <f>Смета!F40</f>
+        <f>Смета!F43</f>
         <v/>
       </c>
       <c r="D8" s="24">
-        <f>IF($C$17=0,0,C8/$C$17)</f>
+        <f>IF($C$16=0,0,C8/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5400,11 +5282,11 @@
         </is>
       </c>
       <c r="C9" s="14">
-        <f>Смета!F51</f>
+        <f>Смета!F54</f>
         <v/>
       </c>
       <c r="D9" s="22">
-        <f>IF($C$17=0,0,C9/$C$17)</f>
+        <f>IF($C$16=0,0,C9/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5418,11 +5300,11 @@
         </is>
       </c>
       <c r="C10" s="9">
-        <f>Смета!F62</f>
+        <f>Смета!F64</f>
         <v/>
       </c>
       <c r="D10" s="24">
-        <f>IF($C$17=0,0,C10/$C$17)</f>
+        <f>IF($C$16=0,0,C10/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5436,11 +5318,11 @@
         </is>
       </c>
       <c r="C11" s="14">
-        <f>Смета!F70</f>
+        <f>Смета!F72</f>
         <v/>
       </c>
       <c r="D11" s="22">
-        <f>IF($C$17=0,0,C11/$C$17)</f>
+        <f>IF($C$16=0,0,C11/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5454,11 +5336,11 @@
         </is>
       </c>
       <c r="C12" s="9">
-        <f>Смета!F78</f>
+        <f>Смета!F80</f>
         <v/>
       </c>
       <c r="D12" s="24">
-        <f>IF($C$17=0,0,C12/$C$17)</f>
+        <f>IF($C$16=0,0,C12/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5472,11 +5354,11 @@
         </is>
       </c>
       <c r="C13" s="14">
-        <f>Смета!F95</f>
+        <f>Смета!F97</f>
         <v/>
       </c>
       <c r="D13" s="22">
-        <f>IF($C$17=0,0,C13/$C$17)</f>
+        <f>IF($C$16=0,0,C13/$C$16)</f>
         <v/>
       </c>
     </row>
@@ -5486,66 +5368,48 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>10. Кухня — встроенное</t>
+          <t>10. Прочее и расходники</t>
         </is>
       </c>
       <c r="C14" s="9">
-        <f>Смета!F103</f>
+        <f>Смета!F104</f>
         <v/>
       </c>
       <c r="D14" s="24">
-        <f>IF($C$17=0,0,C14/$C$17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>11. Прочее и расходники</t>
-        </is>
-      </c>
-      <c r="C15" s="14">
-        <f>Смета!F110</f>
-        <v/>
-      </c>
-      <c r="D15" s="22">
-        <f>IF($C$17=0,0,C15/$C$17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="25" t="n"/>
-      <c r="B17" s="25" t="inlineStr">
+        <f>IF($C$16=0,0,C14/$C$16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="n"/>
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>Итого материалы</t>
         </is>
       </c>
-      <c r="C17" s="26">
-        <f>Смета!F112</f>
-        <v/>
-      </c>
-      <c r="D17" s="27">
-        <f>SUM(D5:D15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="28" t="inlineStr">
-        <is>
-          <t>Не входит в итог: работы; окна; двери; утеплитель и плёнка наружных стен, пола и потолка; каркасы перегородок; любые материалы на террасу. Гарнитур кухни, мебель, шторы, бытовая техника сверх строк 10.4–10.5 — отдельно.</t>
-        </is>
-      </c>
-    </row>
+      <c r="C16" s="26">
+        <f>Смета!F106</f>
+        <v/>
+      </c>
+      <c r="D16" s="27">
+        <f>SUM(D5:D14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Не входит в итог: работы; окна; двери; утеплитель и плёнка наружных стен, пола и потолка; каркасы перегородок; терраса; кухня (гарнитур, мойка, плита, вытяжка). Ламинат кладётся на фанеру 12 мм поверх пластин ТП, не на пластины.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20"/>
     <row r="21"/>
-    <row r="22"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A19:D22"/>
+    <mergeCell ref="A18:D21"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5971,7 +5835,7 @@
     <row r="31">
       <c r="A31" s="34" t="inlineStr">
         <is>
-          <t>Заполнение и обшивка каркасов перегородок</t>
+          <t>Заполнение перегородок минватой; МДФ сразу на обрешётку каркаса. ГВЛВ только в с/у под плитку</t>
         </is>
       </c>
     </row>
@@ -5992,7 +5856,7 @@
     <row r="34">
       <c r="A34" s="34" t="inlineStr">
         <is>
-          <t>Финиш пола: ламинат в жилых, плитка в с/у</t>
+          <t>Пирог пола: черновой настил → пластины ТП → фанера 12 мм → подложка → ламинат; в с/у ГВЛВ + плитка</t>
         </is>
       </c>
     </row>
@@ -6365,7 +6229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6387,7 +6251,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Утеплитель и плёнка уже лежат. Считаем только тёплый пол и финиш.</t>
+          <t>Утеплитель и плёнка уже лежат. Ламинат не на пластины: нужен сплошной настил.</t>
         </is>
       </c>
     </row>
@@ -6622,15 +6486,25 @@
     <row r="15">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>Пирог, который уже сделан: лаги/основание + утеплитель + плёнка. Дальше: теплораспределительные пластины VT.FP.SZ + труба 16 мм + финиш. Под кухонный низ можно не класть пластины (~1.8 м²) — на коробку не влияет.</t>
+          <t>Пирог дальше уже сделанного (лаги + утеплитель + плёнка):
+1) Черновой настил OSB-3 / фанера ФСФ 18 мм по лагам — если под плёнкой ещё дырки между лагами. Если черновой пол уже лежит — эту строку в смете обнулить.
+2) Пластины VT.FP.SZ + труба 16 мм (вкладка Теплый_пол).
+3) Сплошной настил поверх пластин: фанера ФСФ 12 мм в жилых — на НЕЁ кладётся тонкая подложка и ламинат. Прямо на алюминиевые пластины ламинат нельзя: трубы и кромки плит продавят замки.
+4) В с/у поверх труб — 2 слоя ГВЛВ 10 мм, затем гидроизоляция и плитка.
+5) Подложка под ламинат только 1–2 мм «для ТП», без толстой пробки.</t>
         </is>
       </c>
     </row>
     <row r="16"/>
     <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A15:G17"/>
+    <mergeCell ref="A15:G22"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Use 22 mm OSB subfloor and OSB over UFH plates, drop plywood
Laminate still needs a sheet over the plates; that sheet is now OSB-3 12 mm.

Co-authored-by: PavelP78 <PavelP78@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/barnhouse/smeta_barnhouse_mdf.xlsx
+++ b/barnhouse/smeta_barnhouse_mdf.xlsx
@@ -1742,7 +1742,7 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>OSB-3 18 мм / фанера ФСФ 18 мм — черновой настил по лагам</t>
+          <t>OSB-3 22 мм — черновой настил по лагам</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
@@ -1755,7 +1755,7 @@
         <v/>
       </c>
       <c r="E35" s="14" t="n">
-        <v>1650</v>
+        <v>2150</v>
       </c>
       <c r="F35" s="15">
         <f>IF(D35="","",D35*E35)</f>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Саморезы 4.2×55 к лагам</t>
+          <t>Саморезы 4.2×65 к лагам</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -1797,7 +1797,7 @@
         <v>4</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="F36" s="10">
         <f>IF(D36="","",D36*E36)</f>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>черновой настил</t>
+          <t>черновой настил 22 мм</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr"/>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Фанера ФСФ 12 мм поверх пластин ТП — под ламинат</t>
+          <t>OSB-3 12 мм поверх пластин ТП — под ламинат</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
@@ -1832,7 +1832,7 @@
         <v/>
       </c>
       <c r="E37" s="14" t="n">
-        <v>2190</v>
+        <v>1250</v>
       </c>
       <c r="F37" s="15">
         <f>IF(D37="","",D37*E37)</f>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="I37" s="12" t="inlineStr">
         <is>
-          <t>на этот слой: подложка 1–2 мм и ламинат</t>
+          <t>на этот слой: подложка 1–2 мм и ламинат; фанера не закладывается</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Саморезы 3.5×41 + клей по дереву на настил 12 мм</t>
+          <t>Саморезы 3.5×41 + клей по дереву на OSB 12 мм</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
-          <t>фанера жилых + ГВЛВ с/у</t>
+          <t>OSB жилых + ГВЛВ с/у</t>
         </is>
       </c>
       <c r="H39" s="12" t="inlineStr"/>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>класть на фанеру 12 мм, не на пластины</t>
+          <t>класть на OSB 12 мм, не на пластины</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>Пластина VT.FP.SZ.0125 = 1000×125 мм, труба Ø16. Пачка 40 шт. Норма 6.4 шт/м² ≈ 80% покрытия (на петлях пластин нет). Контур не длиннее 80–90 м — отсюда число петель. Пол уже утеплён и под плёнкой: подложку под пластины не закладывал. Сверху на пластины — фанера 12 мм (жилые) / ГВЛВ (с/у), затем финиш. Не класть ламинат на пластины.</t>
+          <t>Пластина VT.FP.SZ.0125 = 1000×125 мм, труба Ø16. Пачка 40 шт. Норма 6.4 шт/м² ≈ 80% покрытия (на петлях пластин нет). Контур не длиннее 80–90 м — отсюда число петель. Пол уже утеплён и под плёнкой: подложку под пластины не закладывал. Сверху на пластины — OSB-3 12 мм (жилые) / ГВЛВ (с/у), затем финиш. Не класть ламинат на пластины.</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5399,7 @@
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>
-          <t>Не входит в итог: работы; окна; двери; утеплитель и плёнка наружных стен, пола и потолка; каркасы перегородок; терраса; кухня (гарнитур, мойка, плита, вытяжка). Ламинат кладётся на фанеру 12 мм поверх пластин ТП, не на пластины.</t>
+          <t>Не входит в итог: работы; окна; двери; утеплитель и плёнка наружных стен, пола и потолка; каркасы перегородок; терраса; кухня (гарнитур, мойка, плита, вытяжка). Ламинат кладётся на OSB-3 12 мм поверх пластин ТП, не на пластины. Фанеры нет.</t>
         </is>
       </c>
     </row>
@@ -5856,7 +5856,7 @@
     <row r="34">
       <c r="A34" s="34" t="inlineStr">
         <is>
-          <t>Пирог пола: черновой настил → пластины ТП → фанера 12 мм → подложка → ламинат; в с/у ГВЛВ + плитка</t>
+          <t>Пирог пола: OSB-3 22 мм → пластины ТП → OSB-3 12 мм → подложка → ламинат; в с/у ГВЛВ + плитка</t>
         </is>
       </c>
     </row>
@@ -6487,9 +6487,9 @@
       <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Пирог дальше уже сделанного (лаги + утеплитель + плёнка):
-1) Черновой настил OSB-3 / фанера ФСФ 18 мм по лагам — если под плёнкой ещё дырки между лагами. Если черновой пол уже лежит — эту строку в смете обнулить.
+1) Черновой настил OSB-3 22 мм по лагам — если под плёнкой ещё дырки между лагами. Если черновой пол уже лежит — эту строку в смете обнулить.
 2) Пластины VT.FP.SZ + труба 16 мм (вкладка Теплый_пол).
-3) Сплошной настил поверх пластин: фанера ФСФ 12 мм в жилых — на НЕЁ кладётся тонкая подложка и ламинат. Прямо на алюминиевые пластины ламинат нельзя: трубы и кромки плит продавят замки.
+3) Второй слой OSB-3 12 мм поверх пластин в жилых — на НЕГО кладётся тонкая подложка и ламинат. Фанера не нужна: OSB дешевле и тот же сплошной щит. Прямо на пластины ламинат нельзя.
 4) В с/у поверх труб — 2 слоя ГВЛВ 10 мм, затем гидроизоляция и плитка.
 5) Подложка под ламинат только 1–2 мм «для ТП», без толстой пробки.</t>
         </is>

</xml_diff>

<commit_message>
Add radiator-heating estimate variant
Same barnhouse materials takeoff with electric radiators instead of
dry UFH, boiler, and the extra OSB layer over plates.

Co-authored-by: PavelP78 <PavelP78@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/barnhouse/smeta_barnhouse_mdf.xlsx
+++ b/barnhouse/smeta_barnhouse_mdf.xlsx
@@ -3176,7 +3176,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>свет, розетки, стиралка, котёл, бойлер</t>
+          <t>свет, розетки, стиралка, бойлер, котёл</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t>Кабель ВВГнг-LS 3×4 (котёл / бойлер)</t>
+          <t>Кабель ВВГнг-LS 3×4 (бойлер)</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
@@ -3794,7 +3794,7 @@
     <row r="108">
       <c r="A108" s="20" t="inlineStr">
         <is>
-          <t>Как пользоваться: меняйте столбец «Цена, ₽» — сумма раздела и итог пересчитаются. Количество с формулой тянется с вкладок Полы / Стены / Потолки / Обшивка / Теплый_пол / С_у. Строки техники (котёл, бойлер) обнулите в «Кол-во», если привезёте своё. Работы, окна, двери, утепление и плёнка наружного контура, каркасы перегородок и вся терраса в смету не входят. Цены — ориентир Петрович СПб / Valtec, сентябрь 2026; перед закупкой сверьте карточку товара. Отделка: МДФ дуб альпийский 2600×238×6 (Союз), без лака — покрытие уже на панели. Кухня (гарнитур, мойка, плита, вытяжка, смеситель) в смету не входит.</t>
+          <t>Как пользоваться: меняйте столбец «Цена, ₽» — сумма раздела и итог пересчитаются. Количество с формулой тянется с вкладок Полы / Стены / Потолки / Обшивка / С_у. Строки техники (котёл, бойлер) обнулите в «Кол-во», если привезёте своё. Работы, окна, двери, утепление и плёнка наружного контура, каркасы перегородок и вся терраса в смету не входят. Цены — ориентир Петрович СПб / Valtec, сентябрь 2026; перед закупкой сверьте карточку товара. Отделка: МДФ дуб альпийский 2600×238×6 (Союз), без лака — покрытие уже на панели. Кухня (гарнитур, мойка, плита, вытяжка, смеситель) в смету не входит.</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
         </is>
       </c>
       <c r="B15" s="39">
-        <f>Теплый_пол!D12</f>
+        <f>Теплый_пол!B12</f>
         <v/>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="E10" s="35" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>нет / не трогаем</t>
         </is>
       </c>
       <c r="F10" s="35" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Контур ТП</t>
+          <t>Отопление пола</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">

</xml_diff>